<commit_message>
feat: implementar script de evaluación NLP con BERTScore y dashboard directivo
</commit_message>
<xml_diff>
--- a/Comparativa_Final_Humano_vs_LLM_v5.xlsx
+++ b/Comparativa_Final_Humano_vs_LLM_v5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\MEGADAPT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_74A5FA1A977DBAAFEB19A0F6455DCE3AB7C64E31" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69546491-AF4A-4BCC-B9A2-1B2012D3584A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1174,6 +1174,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{6CAF4E90-7E91-48FD-A187-F7A25C2CB255}">
+  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;dbae2696-07df-4228-92b1-6ac2906a0e77&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I19"/>

</xml_diff>